<commit_message>
Add game state manager with modState VBA module and GameState sheet
- vba/modState.bas: Full state management module with:
  - Stat get/set/modify with automatic clamping (0..Max)
  - Derived stats (Control, Threat, TransformRisk)
  - Boolean/string/numeric flag system with HasFlag truthiness check
  - Scene history stack with push/pop for Back button support
  - Action log for replay/debug (timestamped entries)
  - Save/load to hidden GameState sheet
  - Snapshot/restore for stack-based undo/rewind
  - State dump for debugging
  - Death (HP<=0) and beast (Humanity<=0) state checks
- build_game_state.py: Python script to initialize the GameState sheet
  with 14 default stats across 5 sections (Stats, Flags, History, Log, Meta)
- GameState sheet added to workbook (hidden)

https://claude.ai/code/session_01FamWb49s4vMEcWYQyfS6mZ
</commit_message>
<xml_diff>
--- a/BloodMoonProtocol_RPG.xlsx
+++ b/BloodMoonProtocol_RPG.xlsx
@@ -26,6 +26,7 @@
     <sheet name="ENDING_VICTORY" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="ENDING_PYRRHIC" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="ENDING_BEAST" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="GameState" sheetId="20" state="hidden" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SceneDB'!$A$1:$R$20</definedName>
@@ -37,7 +38,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -210,8 +211,14 @@
       <name val="Consolas"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="00CCCCCC"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -277,6 +284,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="002D2D2D"/>
         <bgColor rgb="002D2D2D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008B0000"/>
+        <bgColor rgb="008B0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00333333"/>
+        <bgColor rgb="00333333"/>
       </patternFill>
     </fill>
   </fills>
@@ -1215,7 +1234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1397,6 +1416,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="74" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="83" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="84" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="85" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="85" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="85" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -16619,6 +16641,291 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="109" t="inlineStr">
+        <is>
+          <t>STATS</t>
+        </is>
+      </c>
+      <c r="D1" s="109" t="inlineStr">
+        <is>
+          <t>FLAGS</t>
+        </is>
+      </c>
+      <c r="G1" s="109" t="inlineStr">
+        <is>
+          <t>HISTORY</t>
+        </is>
+      </c>
+      <c r="L1" s="109" t="inlineStr">
+        <is>
+          <t>ACTION LOG</t>
+        </is>
+      </c>
+      <c r="Q1" s="109" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="110" t="inlineStr">
+        <is>
+          <t>StatName</t>
+        </is>
+      </c>
+      <c r="B2" s="110" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D2" s="110" t="inlineStr">
+        <is>
+          <t>FlagName</t>
+        </is>
+      </c>
+      <c r="E2" s="110" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G2" s="110" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="H2" s="110" t="inlineStr">
+        <is>
+          <t>SceneID</t>
+        </is>
+      </c>
+      <c r="I2" s="110" t="inlineStr">
+        <is>
+          <t>Choice</t>
+        </is>
+      </c>
+      <c r="J2" s="110" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="L2" s="110" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="M2" s="110" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="N2" s="110" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="O2" s="110" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="Q2" s="110" t="inlineStr">
+        <is>
+          <t>CurrentScene</t>
+        </is>
+      </c>
+      <c r="R2" s="110" t="inlineStr">
+        <is>
+          <t>SaveSlot</t>
+        </is>
+      </c>
+      <c r="S2" s="110" t="inlineStr">
+        <is>
+          <t>SaveTimestamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="111" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="B3" s="111" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q3" s="111" t="inlineStr">
+        <is>
+          <t>TITLE</t>
+        </is>
+      </c>
+      <c r="R3" s="111" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="111" t="inlineStr">
+        <is>
+          <t>MaxHP</t>
+        </is>
+      </c>
+      <c r="B4" s="111" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="111" t="inlineStr">
+        <is>
+          <t>Humanity</t>
+        </is>
+      </c>
+      <c r="B5" s="111" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="111" t="inlineStr">
+        <is>
+          <t>MaxHumanity</t>
+        </is>
+      </c>
+      <c r="B6" s="111" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="111" t="inlineStr">
+        <is>
+          <t>Rage</t>
+        </is>
+      </c>
+      <c r="B7" s="111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="111" t="inlineStr">
+        <is>
+          <t>MaxRage</t>
+        </is>
+      </c>
+      <c r="B8" s="111" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="111" t="inlineStr">
+        <is>
+          <t>Hunger</t>
+        </is>
+      </c>
+      <c r="B9" s="111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="111" t="inlineStr">
+        <is>
+          <t>MaxHunger</t>
+        </is>
+      </c>
+      <c r="B10" s="111" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="111" t="inlineStr">
+        <is>
+          <t>ScentLevel</t>
+        </is>
+      </c>
+      <c r="B11" s="111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="111" t="inlineStr">
+        <is>
+          <t>Suspicion</t>
+        </is>
+      </c>
+      <c r="B12" s="111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="111" t="inlineStr">
+        <is>
+          <t>SilverItems</t>
+        </is>
+      </c>
+      <c r="B13" s="111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="111" t="inlineStr">
+        <is>
+          <t>MoonPhase</t>
+        </is>
+      </c>
+      <c r="B14" s="111" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="111" t="inlineStr">
+        <is>
+          <t>TimeOfDay</t>
+        </is>
+      </c>
+      <c r="B15" s="111" t="n">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="111" t="inlineStr">
+        <is>
+          <t>TransformStage</t>
+        </is>
+      </c>
+      <c r="B16" s="111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>